<commit_message>
Refresh datasets: All India (15%) from All_India_MBBS_Cutoff_2025; MBBS in Other State updated (126 colleges, 6 states)
</commit_message>
<xml_diff>
--- a/data/MBBS_IN_OTHER_STATE.xlsx
+++ b/data/MBBS_IN_OTHER_STATE.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="136">
   <si>
     <t>College Name</t>
   </si>
@@ -367,45 +367,15 @@
     <t>F.H. Medical College &amp; Hospital, Firozabad, Agra(Muslim Minority)</t>
   </si>
   <si>
-    <t>R D Gardi medical college, Ujjain</t>
-  </si>
-  <si>
-    <t>LNCT Medical College &amp; Sewakunj Hospital Indore</t>
-  </si>
-  <si>
-    <t>Index medical college, indore</t>
-  </si>
-  <si>
     <t>Jaipur National University Institute of Medical Sciences and Resarch Centre, Jagatpura, Jaipur</t>
   </si>
   <si>
     <t>Ananta Institute of Medical Sciences &amp; Research Centre, Rajsamand</t>
   </si>
   <si>
-    <t>Sri aurbundo institute medical science, Indore</t>
-  </si>
-  <si>
-    <t>School of Medical Science, Sri Satya Sai University of Technology and Medical Sceinces, Sehore</t>
-  </si>
-  <si>
-    <t>Sukh Sagar Medical College and Hospital Jabalpur</t>
-  </si>
-  <si>
     <t>American International Institute of Medical Sciences, Bedwas</t>
   </si>
   <si>
-    <t>Ram Krishna Medical College Hospital and Research Centre, Bhopal</t>
-  </si>
-  <si>
-    <t>Amaltas medical college, Dewas</t>
-  </si>
-  <si>
-    <t>RKDF Medical college Hospital &amp; Research Centre Bhopal</t>
-  </si>
-  <si>
-    <t>Mahaveer Institute of Medical Science &amp; Research Bhopal</t>
-  </si>
-  <si>
     <t>National Institute of Medical Science &amp; Research, Jaipur</t>
   </si>
   <si>
@@ -452,9 +422,6 @@
   </si>
   <si>
     <t>Rajasthan</t>
-  </si>
-  <si>
-    <t>Madhya Pradesh</t>
   </si>
 </sst>
 </file>
@@ -786,7 +753,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D137"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -808,7 +775,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C2">
         <v>23923</v>
@@ -822,7 +789,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C3">
         <v>27193</v>
@@ -836,7 +803,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C4">
         <v>29857</v>
@@ -850,7 +817,7 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C5">
         <v>30264</v>
@@ -864,7 +831,7 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C6">
         <v>30886</v>
@@ -878,7 +845,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C7">
         <v>32658</v>
@@ -892,7 +859,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C8">
         <v>33265</v>
@@ -906,7 +873,7 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C9">
         <v>39089</v>
@@ -920,7 +887,7 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C10">
         <v>44842</v>
@@ -934,7 +901,7 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C11">
         <v>46084</v>
@@ -948,7 +915,7 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C12">
         <v>46597</v>
@@ -962,7 +929,7 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C13">
         <v>47199</v>
@@ -976,7 +943,7 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C14">
         <v>49834</v>
@@ -990,7 +957,7 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C15">
         <v>51573</v>
@@ -1004,7 +971,7 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C16">
         <v>54489</v>
@@ -1018,7 +985,7 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C17">
         <v>54956</v>
@@ -1032,7 +999,7 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C18">
         <v>55581</v>
@@ -1046,7 +1013,7 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C19">
         <v>56287</v>
@@ -1060,7 +1027,7 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C20">
         <v>58632</v>
@@ -1074,7 +1041,7 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C21">
         <v>62384</v>
@@ -1088,7 +1055,7 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C22">
         <v>62634</v>
@@ -1102,7 +1069,7 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C23">
         <v>62905</v>
@@ -1116,7 +1083,7 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C24">
         <v>66832</v>
@@ -1130,7 +1097,7 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C25">
         <v>67382</v>
@@ -1144,7 +1111,7 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C26">
         <v>72225</v>
@@ -1158,7 +1125,7 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C27">
         <v>73399</v>
@@ -1172,7 +1139,7 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C28">
         <v>74284</v>
@@ -1186,7 +1153,7 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C29">
         <v>74953</v>
@@ -1200,7 +1167,7 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C30">
         <v>75560</v>
@@ -1214,7 +1181,7 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C31">
         <v>75588</v>
@@ -1228,7 +1195,7 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C32">
         <v>75865</v>
@@ -1242,7 +1209,7 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C33">
         <v>76138</v>
@@ -1256,7 +1223,7 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C34">
         <v>77897</v>
@@ -1270,7 +1237,7 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C35">
         <v>82414</v>
@@ -1284,7 +1251,7 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C36">
         <v>82567</v>
@@ -1298,7 +1265,7 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C37">
         <v>85450</v>
@@ -1312,7 +1279,7 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C38">
         <v>88406</v>
@@ -1326,7 +1293,7 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C39">
         <v>89091</v>
@@ -1340,7 +1307,7 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C40">
         <v>89719</v>
@@ -1354,7 +1321,7 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C41">
         <v>91633</v>
@@ -1368,7 +1335,7 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C42">
         <v>92154</v>
@@ -1382,7 +1349,7 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C43">
         <v>95359</v>
@@ -1396,7 +1363,7 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C44">
         <v>95727</v>
@@ -1410,7 +1377,7 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C45">
         <v>98147</v>
@@ -1424,7 +1391,7 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C46">
         <v>101411</v>
@@ -1438,7 +1405,7 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C47">
         <v>102349</v>
@@ -1452,7 +1419,7 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C48">
         <v>103870</v>
@@ -1466,7 +1433,7 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C49">
         <v>105378</v>
@@ -1480,7 +1447,7 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C50">
         <v>105644</v>
@@ -1494,7 +1461,7 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C51">
         <v>106547</v>
@@ -1508,7 +1475,7 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C52">
         <v>108184</v>
@@ -1522,7 +1489,7 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C53">
         <v>109071</v>
@@ -1536,7 +1503,7 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C54">
         <v>111791</v>
@@ -1550,7 +1517,7 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C55">
         <v>112920</v>
@@ -1564,7 +1531,7 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C56">
         <v>115427</v>
@@ -1578,7 +1545,7 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C57">
         <v>117899</v>
@@ -1592,7 +1559,7 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C58">
         <v>119298</v>
@@ -1606,7 +1573,7 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C59">
         <v>121662</v>
@@ -1620,7 +1587,7 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C60">
         <v>122070</v>
@@ -1634,7 +1601,7 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C61">
         <v>124954</v>
@@ -1648,7 +1615,7 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C62">
         <v>132349</v>
@@ -1662,7 +1629,7 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C63">
         <v>133279</v>
@@ -1676,7 +1643,7 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C64">
         <v>134490</v>
@@ -1690,7 +1657,7 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C65">
         <v>134706</v>
@@ -1704,7 +1671,7 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C66">
         <v>137567</v>
@@ -1718,7 +1685,7 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C67">
         <v>137867</v>
@@ -1732,7 +1699,7 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C68">
         <v>140042</v>
@@ -1746,7 +1713,7 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C69">
         <v>142644</v>
@@ -1760,7 +1727,7 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C70">
         <v>143528</v>
@@ -1774,7 +1741,7 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C71">
         <v>144275</v>
@@ -1788,7 +1755,7 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C72">
         <v>153216</v>
@@ -1802,7 +1769,7 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C73">
         <v>160036</v>
@@ -1816,7 +1783,7 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C74">
         <v>160036</v>
@@ -1830,7 +1797,7 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C75">
         <v>171713</v>
@@ -1844,7 +1811,7 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C76">
         <v>189181</v>
@@ -1858,7 +1825,7 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C77">
         <v>190852</v>
@@ -1872,7 +1839,7 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C78">
         <v>195896</v>
@@ -1886,7 +1853,7 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C79">
         <v>196805</v>
@@ -1900,7 +1867,7 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C80">
         <v>197567</v>
@@ -1914,7 +1881,7 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C81">
         <v>197567</v>
@@ -1928,7 +1895,7 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C82">
         <v>212337</v>
@@ -1942,7 +1909,7 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C83">
         <v>229989</v>
@@ -1956,7 +1923,7 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C84">
         <v>234085</v>
@@ -1970,7 +1937,7 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C85">
         <v>244556</v>
@@ -1984,7 +1951,7 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C86">
         <v>266476</v>
@@ -1998,7 +1965,7 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C87">
         <v>269532</v>
@@ -2012,7 +1979,7 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C88">
         <v>296410</v>
@@ -2026,7 +1993,7 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C89">
         <v>334849</v>
@@ -2040,7 +2007,7 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C90">
         <v>336679</v>
@@ -2054,7 +2021,7 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C91">
         <v>351380</v>
@@ -2068,7 +2035,7 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C92">
         <v>357901</v>
@@ -2082,7 +2049,7 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C93">
         <v>364468</v>
@@ -2096,7 +2063,7 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C94">
         <v>375194</v>
@@ -2110,7 +2077,7 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C95">
         <v>382152</v>
@@ -2124,7 +2091,7 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C96">
         <v>383586</v>
@@ -2138,7 +2105,7 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C97">
         <v>392077</v>
@@ -2152,7 +2119,7 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C98">
         <v>402286</v>
@@ -2166,7 +2133,7 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C99">
         <v>404611</v>
@@ -2180,7 +2147,7 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C100">
         <v>421396</v>
@@ -2194,7 +2161,7 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C101">
         <v>427750</v>
@@ -2208,7 +2175,7 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C102">
         <v>433125</v>
@@ -2222,7 +2189,7 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C103">
         <v>436705</v>
@@ -2236,7 +2203,7 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C104">
         <v>439268</v>
@@ -2250,7 +2217,7 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C105">
         <v>440266</v>
@@ -2264,7 +2231,7 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C106">
         <v>445758</v>
@@ -2278,7 +2245,7 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C107">
         <v>500475</v>
@@ -2292,7 +2259,7 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C108">
         <v>558179</v>
@@ -2306,7 +2273,7 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C109">
         <v>580210</v>
@@ -2320,7 +2287,7 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C110">
         <v>581641</v>
@@ -2334,7 +2301,7 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C111">
         <v>591567</v>
@@ -2348,7 +2315,7 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C112">
         <v>600891</v>
@@ -2362,7 +2329,7 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C113">
         <v>628502</v>
@@ -2376,7 +2343,7 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C114">
         <v>722941</v>
@@ -2390,13 +2357,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C115">
-        <v>739444</v>
+        <v>911481</v>
       </c>
       <c r="D115">
-        <v>214</v>
+        <v>177</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -2404,13 +2371,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C116">
-        <v>780590</v>
+        <v>919665</v>
       </c>
       <c r="D116">
-        <v>205</v>
+        <v>176</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -2418,13 +2385,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C117">
-        <v>894626</v>
+        <v>1001133</v>
       </c>
       <c r="D117">
-        <v>180</v>
+        <v>160</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -2432,13 +2399,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C118">
-        <v>911481</v>
+        <v>1076504</v>
       </c>
       <c r="D118">
-        <v>177</v>
+        <v>147</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -2446,13 +2413,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="C119">
-        <v>919665</v>
+        <v>1085133</v>
       </c>
       <c r="D119">
-        <v>176</v>
+        <v>146</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -2460,13 +2427,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C120">
-        <v>920506</v>
+        <v>1117630</v>
       </c>
       <c r="D120">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -2474,13 +2441,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C121">
-        <v>926271</v>
+        <v>1267561</v>
       </c>
       <c r="D121">
-        <v>174</v>
+        <v>119</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -2488,13 +2455,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C122">
-        <v>940445</v>
+        <v>1268204</v>
       </c>
       <c r="D122">
-        <v>171</v>
+        <v>119</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -2502,13 +2469,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C123">
-        <v>1001133</v>
+        <v>1291243</v>
       </c>
       <c r="D123">
-        <v>160</v>
+        <v>166</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -2516,13 +2483,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C124">
-        <v>1009228</v>
+        <v>1296229</v>
       </c>
       <c r="D124">
-        <v>159</v>
+        <v>116</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -2530,13 +2497,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C125">
-        <v>1037524</v>
+        <v>1307816</v>
       </c>
       <c r="D125">
-        <v>154</v>
+        <v>115</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -2544,13 +2511,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C126">
-        <v>1049504</v>
+        <v>1314408</v>
       </c>
       <c r="D126">
-        <v>152</v>
+        <v>113</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -2558,152 +2525,12 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="C127">
-        <v>1055818</v>
+        <v>6699854</v>
       </c>
       <c r="D127">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4">
-      <c r="A128" t="s">
-        <v>130</v>
-      </c>
-      <c r="B128" t="s">
-        <v>145</v>
-      </c>
-      <c r="C128">
-        <v>1076504</v>
-      </c>
-      <c r="D128">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4">
-      <c r="A129" t="s">
-        <v>131</v>
-      </c>
-      <c r="B129" t="s">
-        <v>144</v>
-      </c>
-      <c r="C129">
-        <v>1085133</v>
-      </c>
-      <c r="D129">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4">
-      <c r="A130" t="s">
-        <v>132</v>
-      </c>
-      <c r="B130" t="s">
-        <v>145</v>
-      </c>
-      <c r="C130">
-        <v>1117630</v>
-      </c>
-      <c r="D130">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4">
-      <c r="A131" t="s">
-        <v>133</v>
-      </c>
-      <c r="B131" t="s">
-        <v>145</v>
-      </c>
-      <c r="C131">
-        <v>1267561</v>
-      </c>
-      <c r="D131">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4">
-      <c r="A132" t="s">
-        <v>134</v>
-      </c>
-      <c r="B132" t="s">
-        <v>145</v>
-      </c>
-      <c r="C132">
-        <v>1268204</v>
-      </c>
-      <c r="D132">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4">
-      <c r="A133" t="s">
-        <v>135</v>
-      </c>
-      <c r="B133" t="s">
-        <v>145</v>
-      </c>
-      <c r="C133">
-        <v>1291243</v>
-      </c>
-      <c r="D133">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4">
-      <c r="A134" t="s">
-        <v>136</v>
-      </c>
-      <c r="B134" t="s">
-        <v>145</v>
-      </c>
-      <c r="C134">
-        <v>1296229</v>
-      </c>
-      <c r="D134">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4">
-      <c r="A135" t="s">
-        <v>137</v>
-      </c>
-      <c r="B135" t="s">
-        <v>145</v>
-      </c>
-      <c r="C135">
-        <v>1307816</v>
-      </c>
-      <c r="D135">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4">
-      <c r="A136" t="s">
-        <v>138</v>
-      </c>
-      <c r="B136" t="s">
-        <v>145</v>
-      </c>
-      <c r="C136">
-        <v>1314408</v>
-      </c>
-      <c r="D136">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4">
-      <c r="A137" t="s">
-        <v>139</v>
-      </c>
-      <c r="B137" t="s">
-        <v>144</v>
-      </c>
-      <c r="C137">
-        <v>6699854</v>
-      </c>
-      <c r="D137">
         <v>231</v>
       </c>
     </row>

</xml_diff>